<commit_message>
Changed the formatting of the name of the resume
</commit_message>
<xml_diff>
--- a/data/invalid_jobs.xlsx
+++ b/data/invalid_jobs.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="42.14285714285715" customWidth="1" min="1" max="2"/>
@@ -2240,221 +2240,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://jobright.ai/jobs/info/6ab1684f32552369083e1eda</t>
+          <t>https://jobright.ai/jobs/info/6ab56a72d85922de20ce0eba</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>ALREADY_APPLIED</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>url:a6a86ab07d8302db8104</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab1879e191d8c340dbdb376</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>OTHER</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>url:f2a22f303cc344dc2767</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab16cccf9692ca98b0497ff</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>url:ac1991fa27bdc6581f0a</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab1b3ded43eb922ca0c0c46</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>url:17a259bd809b985ca26c</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab1d39e23005eee3545cb59</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>NEEDS_SECURITY_CLERANCE</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>url:5b6a65c3c10db2d28240</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab18d25d2a93d5a97ebb548</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>url:7e277abf7b6021a50800</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab13b1bf9692ca98b0483c8</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>OTHER</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>url:0a731d30ef1311f066ef</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6a87694fe8b6601d129037d7</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>OTHER</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>url:ba34ec13c46fa863d246</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab19783191d8c340dbdbab3</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>url:83faa79fe9917db71b6a</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6a31e5440ff23769fdb20f07</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>url:a1b5bf39f1042e2f4cdb</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6a9e9ed22c964816f65edf4a</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>url:f224a7b55a0e026f09cc</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab2c4d230340229a322f9c5</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>url:f5092bdd5006e854fc2e</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>https://jobright.ai/jobs/info/6ab302711e4847ddae917cd5</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>US_CITIZENSHIP_REQUIRED</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>url:23617f1748aa6551e3ec</t>
+          <t>url:7837691e3a86b6e190b1</t>
         </is>
       </c>
     </row>

</xml_diff>